<commit_message>
refactor: 移除 pandas 依赖，使用 openpyxl 直接读取 Excel
- 重写 data_handler.py，用 openpyxl + 纯 Python 替代 pandas
- 重写 selector.py，用 list/dict 替代 DataFrame
- 去掉 main_window.py 中的 PIL 导入（保留 pillow 供 ttkbootstrap 使用）
- 可执行文件体积从 42MB 缩减至 22MB（减少 48%）
- 更新版本号至 1.2.0
</commit_message>
<xml_diff>
--- a/data/test_data.xlsx
+++ b/data/test_data.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,12 +442,20 @@
           <t>成绩</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>是否班委</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>是否团员</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2023001</t>
-        </is>
+      <c r="A2" t="n">
+        <v>2023001</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -467,12 +475,20 @@
       <c r="E2" t="n">
         <v>85</v>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2023002</t>
-        </is>
+      <c r="A3" t="n">
+        <v>2023002</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -492,12 +508,20 @@
       <c r="E3" t="n">
         <v>92</v>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2023003</t>
-        </is>
+      <c r="A4" t="n">
+        <v>2023003</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -517,12 +541,20 @@
       <c r="E4" t="n">
         <v>78</v>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2023004</t>
-        </is>
+      <c r="A5" t="n">
+        <v>2023004</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -542,12 +574,20 @@
       <c r="E5" t="n">
         <v>95</v>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2023005</t>
-        </is>
+      <c r="A6" t="n">
+        <v>2023005</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -566,6 +606,181 @@
       </c>
       <c r="E6" t="n">
         <v>88</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2023006</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>孙八</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>女</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>1班</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>90</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2023007</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>周九</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>男</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1班</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>76</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2023008</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>吴十</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>女</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2班</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>82</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2023009</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>郑一</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>男</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>1班</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>88</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2023010</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>王二</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>女</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2班</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>91</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>